<commit_message>
Avances 15/04: continuación iteraciones
</commit_message>
<xml_diff>
--- a/Códigos_oficiales/codigos_optimizacion/hiperparametros/resultados_cv_pso_20260408_171225/cv_fold_results - copia 1.xlsx
+++ b/Códigos_oficiales/codigos_optimizacion/hiperparametros/resultados_cv_pso_20260408_171225/cv_fold_results - copia 1.xlsx
@@ -8,52 +8,261 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Códigos_oficiales\codigos_optimizacion\hiperparametros\resultados_cv_pso_20260408_171225\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43413C0-78A7-4B9D-BDFD-8BBD4975FD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01988514-0FD9-4C69-BECB-A1E585F916F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="3" r:id="rId2"/>
+    <sheet name="Hoja2 (2)" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$1</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">Hoja2!$B$12:$B$16</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Hoja2!$B$17:$B$21</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Hoja2!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Hoja2!$D$17:$D$21</definedName>
     <definedName name="_xlchart.v1.10" hidden="1">Hoja2!$F$2</definedName>
+    <definedName name="_xlchart.v1.100" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.101" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.102" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.103" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.104" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.105" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.106" hidden="1">'Hoja2 (2)'!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.107" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.108" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.109" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
     <definedName name="_xlchart.v1.11" hidden="1">Hoja2!$F$3</definedName>
+    <definedName name="_xlchart.v1.110" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.111" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.112" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.113" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.114" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.115" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.116" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.117" hidden="1">'Hoja2 (2)'!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.118" hidden="1">'Hoja2 (2)'!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.119" hidden="1">'Hoja2 (2)'!$C$42:$C$46</definedName>
     <definedName name="_xlchart.v1.12" hidden="1">Hoja2!$F$4</definedName>
+    <definedName name="_xlchart.v1.120" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.121" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.122" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.123" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.124" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.125" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.126" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.127" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.128" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.129" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
     <definedName name="_xlchart.v1.13" hidden="1">Hoja2!$F$5</definedName>
+    <definedName name="_xlchart.v1.130" hidden="1">'Hoja2 (2)'!$F$1</definedName>
+    <definedName name="_xlchart.v1.131" hidden="1">'Hoja2 (2)'!$F$2:$F$10</definedName>
+    <definedName name="_xlchart.v1.132" hidden="1">'Hoja2 (2)'!$G$1</definedName>
+    <definedName name="_xlchart.v1.133" hidden="1">'Hoja2 (2)'!$G$2:$G$10</definedName>
+    <definedName name="_xlchart.v1.134" hidden="1">'Hoja2 (2)'!$H$1</definedName>
+    <definedName name="_xlchart.v1.135" hidden="1">'Hoja2 (2)'!$H$2:$H$10</definedName>
+    <definedName name="_xlchart.v1.136" hidden="1">'Hoja2 (2)'!$I$1</definedName>
+    <definedName name="_xlchart.v1.137" hidden="1">'Hoja2 (2)'!$I$2:$I$10</definedName>
+    <definedName name="_xlchart.v1.138" hidden="1">'Hoja2 (2)'!$J$1</definedName>
+    <definedName name="_xlchart.v1.139" hidden="1">'Hoja2 (2)'!$J$2:$J$10</definedName>
     <definedName name="_xlchart.v1.14" hidden="1">Hoja2!$F$6</definedName>
+    <definedName name="_xlchart.v1.140" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.141" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.142" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.143" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.144" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.145" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.146" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.147" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.148" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.149" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
     <definedName name="_xlchart.v1.15" hidden="1">Hoja2!$F$7</definedName>
+    <definedName name="_xlchart.v1.150" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.151" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.152" hidden="1">'Hoja2 (2)'!$F$1</definedName>
+    <definedName name="_xlchart.v1.153" hidden="1">'Hoja2 (2)'!$F$2:$F$10</definedName>
+    <definedName name="_xlchart.v1.154" hidden="1">'Hoja2 (2)'!$G$1</definedName>
+    <definedName name="_xlchart.v1.155" hidden="1">'Hoja2 (2)'!$G$2:$G$10</definedName>
+    <definedName name="_xlchart.v1.156" hidden="1">'Hoja2 (2)'!$H$1</definedName>
+    <definedName name="_xlchart.v1.157" hidden="1">'Hoja2 (2)'!$H$2:$H$10</definedName>
+    <definedName name="_xlchart.v1.158" hidden="1">'Hoja2 (2)'!$I$1</definedName>
+    <definedName name="_xlchart.v1.159" hidden="1">'Hoja2 (2)'!$I$2:$I$10</definedName>
     <definedName name="_xlchart.v1.16" hidden="1">Hoja2!$F$8</definedName>
+    <definedName name="_xlchart.v1.160" hidden="1">'Hoja2 (2)'!$J$1</definedName>
+    <definedName name="_xlchart.v1.161" hidden="1">'Hoja2 (2)'!$J$2:$J$10</definedName>
+    <definedName name="_xlchart.v1.162" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.163" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.164" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.165" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.166" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.167" hidden="1">'Hoja2 (2)'!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.168" hidden="1">'Hoja2 (2)'!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.169" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
     <definedName name="_xlchart.v1.17" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">Hoja2!$D$12:$D$16</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">Hoja2!$D$17:$D$21</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Hoja2!$B$22:$B$26</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">Hoja2!$D$22:$D$26</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">Hoja2!$D$27:$D$31</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">Hoja2!$D$2:$D$6</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">Hoja2!$D$32:$D$36</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">Hoja2!$D$37:$D$41</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">Hoja2!$D$42:$D$46</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">Hoja2!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.170" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.171" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.172" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.173" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.174" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.175" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.176" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.177" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.178" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.179" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Hoja2!$B$12:$B$16</definedName>
+    <definedName name="_xlchart.v1.180" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.181" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.182" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.183" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.184" hidden="1">'Hoja2 (2)'!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.185" hidden="1">'Hoja2 (2)'!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.186" hidden="1">'Hoja2 (2)'!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.187" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.188" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.189" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Hoja2!$B$17:$B$21</definedName>
+    <definedName name="_xlchart.v1.190" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.191" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.192" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.193" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.194" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.195" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.196" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.197" hidden="1">'Hoja2 (2)'!$F$1</definedName>
+    <definedName name="_xlchart.v1.198" hidden="1">'Hoja2 (2)'!$F$2:$F$10</definedName>
+    <definedName name="_xlchart.v1.199" hidden="1">'Hoja2 (2)'!$G$1</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Hoja2!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">Hoja2!$B$22:$B$26</definedName>
+    <definedName name="_xlchart.v1.200" hidden="1">'Hoja2 (2)'!$G$2:$G$10</definedName>
+    <definedName name="_xlchart.v1.201" hidden="1">'Hoja2 (2)'!$H$1</definedName>
+    <definedName name="_xlchart.v1.202" hidden="1">'Hoja2 (2)'!$H$2:$H$10</definedName>
+    <definedName name="_xlchart.v1.203" hidden="1">'Hoja2 (2)'!$I$1</definedName>
+    <definedName name="_xlchart.v1.204" hidden="1">'Hoja2 (2)'!$I$2:$I$10</definedName>
+    <definedName name="_xlchart.v1.205" hidden="1">'Hoja2 (2)'!$J$1</definedName>
+    <definedName name="_xlchart.v1.206" hidden="1">'Hoja2 (2)'!$J$2:$J$10</definedName>
+    <definedName name="_xlchart.v1.207" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.208" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.209" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">Hoja2!$B$27:$B$31</definedName>
+    <definedName name="_xlchart.v1.210" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.211" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.212" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.213" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.214" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.215" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.216" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.217" hidden="1">'Hoja2 (2)'!$F$10</definedName>
+    <definedName name="_xlchart.v1.218" hidden="1">'Hoja2 (2)'!$F$2</definedName>
+    <definedName name="_xlchart.v1.219" hidden="1">'Hoja2 (2)'!$F$3</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">Hoja2!$B$2:$B$6</definedName>
+    <definedName name="_xlchart.v1.220" hidden="1">'Hoja2 (2)'!$F$4</definedName>
+    <definedName name="_xlchart.v1.221" hidden="1">'Hoja2 (2)'!$F$5</definedName>
+    <definedName name="_xlchart.v1.222" hidden="1">'Hoja2 (2)'!$F$6</definedName>
+    <definedName name="_xlchart.v1.223" hidden="1">'Hoja2 (2)'!$F$7</definedName>
+    <definedName name="_xlchart.v1.224" hidden="1">'Hoja2 (2)'!$F$8</definedName>
+    <definedName name="_xlchart.v1.225" hidden="1">'Hoja2 (2)'!$F$9</definedName>
+    <definedName name="_xlchart.v1.226" hidden="1">'Hoja2 (2)'!$B$12:$B$16</definedName>
+    <definedName name="_xlchart.v1.227" hidden="1">'Hoja2 (2)'!$B$17:$B$21</definedName>
+    <definedName name="_xlchart.v1.228" hidden="1">'Hoja2 (2)'!$B$22:$B$26</definedName>
+    <definedName name="_xlchart.v1.229" hidden="1">'Hoja2 (2)'!$B$27:$B$31</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">Hoja2!$B$32:$B$36</definedName>
+    <definedName name="_xlchart.v1.230" hidden="1">'Hoja2 (2)'!$B$2:$B$6</definedName>
+    <definedName name="_xlchart.v1.231" hidden="1">'Hoja2 (2)'!$B$32:$B$36</definedName>
+    <definedName name="_xlchart.v1.232" hidden="1">'Hoja2 (2)'!$B$37:$B$41</definedName>
+    <definedName name="_xlchart.v1.233" hidden="1">'Hoja2 (2)'!$B$42:$B$46</definedName>
+    <definedName name="_xlchart.v1.234" hidden="1">'Hoja2 (2)'!$B$7:$B$11</definedName>
+    <definedName name="_xlchart.v1.235" hidden="1">'Hoja2 (2)'!$F$10</definedName>
+    <definedName name="_xlchart.v1.236" hidden="1">'Hoja2 (2)'!$F$2</definedName>
+    <definedName name="_xlchart.v1.237" hidden="1">'Hoja2 (2)'!$F$3</definedName>
+    <definedName name="_xlchart.v1.238" hidden="1">'Hoja2 (2)'!$F$4</definedName>
+    <definedName name="_xlchart.v1.239" hidden="1">'Hoja2 (2)'!$F$5</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">Hoja2!$B$37:$B$41</definedName>
+    <definedName name="_xlchart.v1.240" hidden="1">'Hoja2 (2)'!$F$6</definedName>
+    <definedName name="_xlchart.v1.241" hidden="1">'Hoja2 (2)'!$F$7</definedName>
+    <definedName name="_xlchart.v1.242" hidden="1">'Hoja2 (2)'!$F$8</definedName>
+    <definedName name="_xlchart.v1.243" hidden="1">'Hoja2 (2)'!$F$9</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">Hoja2!$B$42:$B$46</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">Hoja2!$B$7:$B$11</definedName>
     <definedName name="_xlchart.v1.27" hidden="1">Hoja2!$F$10</definedName>
     <definedName name="_xlchart.v1.28" hidden="1">Hoja2!$F$2</definedName>
     <definedName name="_xlchart.v1.29" hidden="1">Hoja2!$F$3</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Hoja2!$B$27:$B$31</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Hoja2!$D$27:$D$31</definedName>
     <definedName name="_xlchart.v1.30" hidden="1">Hoja2!$F$4</definedName>
     <definedName name="_xlchart.v1.31" hidden="1">Hoja2!$F$5</definedName>
     <definedName name="_xlchart.v1.32" hidden="1">Hoja2!$F$6</definedName>
     <definedName name="_xlchart.v1.33" hidden="1">Hoja2!$F$7</definedName>
     <definedName name="_xlchart.v1.34" hidden="1">Hoja2!$F$8</definedName>
     <definedName name="_xlchart.v1.35" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Hoja2!$B$2:$B$6</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Hoja2!$B$32:$B$36</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Hoja2!$B$37:$B$41</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Hoja2!$B$42:$B$46</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Hoja2!$B$7:$B$11</definedName>
+    <definedName name="_xlchart.v1.36" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.37" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.38" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.39" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Hoja2!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.40" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.41" hidden="1">'Hoja2 (2)'!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.42" hidden="1">'Hoja2 (2)'!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.43" hidden="1">'Hoja2 (2)'!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.44" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.45" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.46" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.47" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.48" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.49" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Hoja2!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.50" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.51" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.52" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.53" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.54" hidden="1">'Hoja2 (2)'!$F$1</definedName>
+    <definedName name="_xlchart.v1.55" hidden="1">'Hoja2 (2)'!$F$2:$F$10</definedName>
+    <definedName name="_xlchart.v1.56" hidden="1">'Hoja2 (2)'!$G$1</definedName>
+    <definedName name="_xlchart.v1.57" hidden="1">'Hoja2 (2)'!$G$2:$G$10</definedName>
+    <definedName name="_xlchart.v1.58" hidden="1">'Hoja2 (2)'!$H$1</definedName>
+    <definedName name="_xlchart.v1.59" hidden="1">'Hoja2 (2)'!$H$2:$H$10</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Hoja2!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.60" hidden="1">'Hoja2 (2)'!$I$1</definedName>
+    <definedName name="_xlchart.v1.61" hidden="1">'Hoja2 (2)'!$I$2:$I$10</definedName>
+    <definedName name="_xlchart.v1.62" hidden="1">'Hoja2 (2)'!$J$1</definedName>
+    <definedName name="_xlchart.v1.63" hidden="1">'Hoja2 (2)'!$J$2:$J$10</definedName>
+    <definedName name="_xlchart.v1.64" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.65" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.66" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.67" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.68" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.69" hidden="1">'Hoja2 (2)'!$C$32:$C$36</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Hoja2!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.70" hidden="1">'Hoja2 (2)'!$C$37:$C$41</definedName>
+    <definedName name="_xlchart.v1.71" hidden="1">'Hoja2 (2)'!$C$42:$C$46</definedName>
+    <definedName name="_xlchart.v1.72" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.73" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.74" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
+    <definedName name="_xlchart.v1.75" hidden="1">'Hoja2 (2)'!$D$22:$D$26</definedName>
+    <definedName name="_xlchart.v1.76" hidden="1">'Hoja2 (2)'!$D$27:$D$31</definedName>
+    <definedName name="_xlchart.v1.77" hidden="1">'Hoja2 (2)'!$D$2:$D$6</definedName>
+    <definedName name="_xlchart.v1.78" hidden="1">'Hoja2 (2)'!$D$32:$D$36</definedName>
+    <definedName name="_xlchart.v1.79" hidden="1">'Hoja2 (2)'!$D$37:$D$41</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Hoja2!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.80" hidden="1">'Hoja2 (2)'!$D$42:$D$46</definedName>
+    <definedName name="_xlchart.v1.81" hidden="1">'Hoja2 (2)'!$D$7:$D$11</definedName>
+    <definedName name="_xlchart.v1.82" hidden="1">'Hoja2 (2)'!$F$1</definedName>
+    <definedName name="_xlchart.v1.83" hidden="1">'Hoja2 (2)'!$F$2:$F$10</definedName>
+    <definedName name="_xlchart.v1.84" hidden="1">'Hoja2 (2)'!$G$1</definedName>
+    <definedName name="_xlchart.v1.85" hidden="1">'Hoja2 (2)'!$G$2:$G$10</definedName>
+    <definedName name="_xlchart.v1.86" hidden="1">'Hoja2 (2)'!$H$1</definedName>
+    <definedName name="_xlchart.v1.87" hidden="1">'Hoja2 (2)'!$H$2:$H$10</definedName>
+    <definedName name="_xlchart.v1.88" hidden="1">'Hoja2 (2)'!$I$1</definedName>
+    <definedName name="_xlchart.v1.89" hidden="1">'Hoja2 (2)'!$I$2:$I$10</definedName>
     <definedName name="_xlchart.v1.9" hidden="1">Hoja2!$F$10</definedName>
+    <definedName name="_xlchart.v1.90" hidden="1">'Hoja2 (2)'!$J$1</definedName>
+    <definedName name="_xlchart.v1.91" hidden="1">'Hoja2 (2)'!$J$2:$J$10</definedName>
+    <definedName name="_xlchart.v1.92" hidden="1">'Hoja2 (2)'!$C$12:$C$16</definedName>
+    <definedName name="_xlchart.v1.93" hidden="1">'Hoja2 (2)'!$C$17:$C$21</definedName>
+    <definedName name="_xlchart.v1.94" hidden="1">'Hoja2 (2)'!$C$22:$C$26</definedName>
+    <definedName name="_xlchart.v1.95" hidden="1">'Hoja2 (2)'!$C$27:$C$31</definedName>
+    <definedName name="_xlchart.v1.96" hidden="1">'Hoja2 (2)'!$C$2:$C$6</definedName>
+    <definedName name="_xlchart.v1.97" hidden="1">'Hoja2 (2)'!$C$7:$C$11</definedName>
+    <definedName name="_xlchart.v1.98" hidden="1">'Hoja2 (2)'!$D$12:$D$16</definedName>
+    <definedName name="_xlchart.v1.99" hidden="1">'Hoja2 (2)'!$D$17:$D$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -73,7 +282,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="75">
   <si>
     <t>combo_id</t>
   </si>
@@ -627,6 +836,212 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
+        <cx:f>_xlchart.v1.22</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.26</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.18</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="3">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.19</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="4">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.20</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="5">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.21</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="6">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.23</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="7">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.24</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="8">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.25</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Train cost</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Train cost</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{AC52099B-95EA-4C1C-A908-DFA93BE74B1E}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.28</cx:f>
+              <cx:v>1</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000001-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.29</cx:f>
+              <cx:v>2</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000002-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.30</cx:f>
+              <cx:v>3</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000003-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.31</cx:f>
+              <cx:v>4</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="3"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000004-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.32</cx:f>
+              <cx:v>5</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="4"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000005-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.33</cx:f>
+              <cx:v>6</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="5"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000006-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.34</cx:f>
+              <cx:v>7</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="6"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000007-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.35</cx:f>
+              <cx:v>8</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="7"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000008-9A62-4DBD-8E01-86C3D71B49FF}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.27</cx:f>
+              <cx:v>9</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="8"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling max="0.16000000000000003"/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+        <cx:numFmt formatCode="0,000" sourceLinked="0"/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
         <cx:f>_xlchart.v1.4</cx:f>
       </cx:numDim>
     </cx:data>
@@ -675,7 +1090,7 @@
     <cx:title pos="t" align="ctr" overlay="0">
       <cx:tx>
         <cx:txData>
-          <cx:v>Train cost</cx:v>
+          <cx:v>Validation cost</cx:v>
         </cx:txData>
       </cx:tx>
       <cx:txPr>
@@ -695,7 +1110,7 @@
               </a:solidFill>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>Train cost</a:t>
+            <a:t>Validation cost</a:t>
           </a:r>
         </a:p>
       </cx:txPr>
@@ -828,104 +1243,118 @@
 </cx:chartSpace>
 </file>
 
-<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.22</cx:f>
+        <cx:f>_xlchart.v1.68</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.26</cx:f>
+        <cx:f>_xlchart.v1.77</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.18</cx:f>
+        <cx:f>_xlchart.v1.72</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.19</cx:f>
+        <cx:f>_xlchart.v1.81</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="4">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.20</cx:f>
+        <cx:f>_xlchart.v1.64</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="5">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.21</cx:f>
+        <cx:f>_xlchart.v1.73</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="6">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.23</cx:f>
+        <cx:f>_xlchart.v1.65</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="7">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.24</cx:f>
+        <cx:f>_xlchart.v1.74</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="8">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.25</cx:f>
+        <cx:f>_xlchart.v1.66</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="9">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.75</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="10">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.67</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="11">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.76</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="12">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.69</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="13">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.78</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="14">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.70</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="15">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.79</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="16">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.71</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="17">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.80</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
   <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0">
-      <cx:tx>
-        <cx:txData>
-          <cx:v>Validation cost</cx:v>
-        </cx:txData>
-      </cx:tx>
-      <cx:txPr>
-        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Validation cost</a:t>
-          </a:r>
-        </a:p>
-      </cx:txPr>
-    </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
-        <cx:series layoutId="boxWhisker" uniqueId="{AC52099B-95EA-4C1C-A908-DFA93BE74B1E}">
+        <cx:series layoutId="boxWhisker" uniqueId="{00000005-DEDA-4B95-B354-5AEABB406134}" formatIdx="0">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.28</cx:f>
-              <cx:v>1</cx:v>
+              <cx:v>1 train cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="0"/>
           <cx:layoutPr>
-            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000001-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{00000006-DEDA-4B95-B354-5AEABB406134}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.29</cx:f>
-              <cx:v>2</cx:v>
+              <cx:v>1 val cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="1"/>
@@ -933,11 +1362,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000002-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{00000008-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.30</cx:f>
-              <cx:v>3</cx:v>
+              <cx:v>2 train cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="2"/>
@@ -945,11 +1373,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000003-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{00000009-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.31</cx:f>
-              <cx:v>4</cx:v>
+              <cx:v>2 val cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="3"/>
@@ -957,11 +1384,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000004-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000A-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.32</cx:f>
-              <cx:v>5</cx:v>
+              <cx:v>3 train cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="4"/>
@@ -969,11 +1395,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000005-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000B-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.33</cx:f>
-              <cx:v>6</cx:v>
+              <cx:v>3 val cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="5"/>
@@ -981,11 +1406,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000006-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000C-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.34</cx:f>
-              <cx:v>7</cx:v>
+              <cx:v>4 train cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="6"/>
@@ -993,11 +1417,10 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000007-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000D-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.35</cx:f>
-              <cx:v>8</cx:v>
+              <cx:v>4 val cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="7"/>
@@ -1005,14 +1428,112 @@
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
         </cx:series>
-        <cx:series layoutId="boxWhisker" uniqueId="{00000008-9A62-4DBD-8E01-86C3D71B49FF}">
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000E-DEDA-4B95-B354-5AEABB406134}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.27</cx:f>
-              <cx:v>9</cx:v>
+              <cx:v>5 train cost</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:dataId val="8"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{0000000F-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>5 val cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="9"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000010-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>6 train cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="10"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000011-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>6 val cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="11"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000012-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>7 train cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="12"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000013-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>7 val cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="13"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000014-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>8 train cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="14"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000015-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>8 val cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="15"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000016-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>9 train cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="16"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000017-DEDA-4B95-B354-5AEABB406134}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>9 val cost</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="17"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
           </cx:layoutPr>
@@ -1023,10 +1544,13 @@
         <cx:tickLabels/>
       </cx:axis>
       <cx:axis id="1">
-        <cx:valScaling max="0.16000000000000003"/>
+        <cx:valScaling max="0.13200000000000001"/>
         <cx:majorGridlines/>
+        <cx:minorGridlines/>
+        <cx:majorTickMarks type="cross"/>
+        <cx:minorTickMarks type="cross"/>
         <cx:tickLabels/>
-        <cx:numFmt formatCode="0,000" sourceLinked="0"/>
+        <cx:numFmt formatCode="0,00" sourceLinked="0"/>
       </cx:axis>
     </cx:plotArea>
     <cx:legend pos="b" align="ctr" overlay="0"/>
@@ -1114,6 +1638,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
   <cs:axisTitle>
@@ -1630,6 +2194,521 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2273,6 +3352,89 @@
             <a:xfrm>
               <a:off x="4983480" y="5295900"/>
               <a:ext cx="5158740" cy="3036570"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-CL" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>26670</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Gráfico 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{538DA45C-3FB9-FDB0-D009-AC645B397C4C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4945380" y="2061210"/>
+              <a:ext cx="7239000" cy="4872990"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -5892,4 +7054,897 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8322FCF6-B8A1-4319-BED9-8CE9D116E0E9}">
+  <dimension ref="A1:J46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I1" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="37" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13">
+        <v>3.7092048573396118E-2</v>
+      </c>
+      <c r="C2" s="15">
+        <f>B2/4</f>
+        <v>9.2730121433490294E-3</v>
+      </c>
+      <c r="D2" s="13">
+        <v>1.172093869167079E-2</v>
+      </c>
+      <c r="F2" s="32">
+        <v>1</v>
+      </c>
+      <c r="G2" s="33">
+        <f>AVERAGE(B2:B6)</f>
+        <v>5.4480304603383489E-2</v>
+      </c>
+      <c r="H2" s="34">
+        <f>_xlfn.STDEV.S(B2:B6)</f>
+        <v>5.7432180488516803E-2</v>
+      </c>
+      <c r="I2" s="34">
+        <f>AVERAGE(D2:D6)</f>
+        <v>3.6972600811190179E-2</v>
+      </c>
+      <c r="J2" s="34">
+        <f>_xlfn.STDEV.S(D2:D6)</f>
+        <v>2.2821833575323146E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13">
+        <v>0.15599845269902229</v>
+      </c>
+      <c r="C3" s="15">
+        <f t="shared" ref="C3:C46" si="0">B3/4</f>
+        <v>3.8999613174755574E-2</v>
+      </c>
+      <c r="D3" s="13">
+        <v>2.2900716883617861E-2</v>
+      </c>
+      <c r="F3" s="29">
+        <v>2</v>
+      </c>
+      <c r="G3" s="30">
+        <f>AVERAGE(B7:B11)</f>
+        <v>3.9132291833710704E-2</v>
+      </c>
+      <c r="H3" s="31">
+        <f>_xlfn.STDEV.S(B7:B11)</f>
+        <v>1.1042932191310369E-2</v>
+      </c>
+      <c r="I3" s="31">
+        <f>AVERAGE(D7:D11)</f>
+        <v>1.3536307887529056E-2</v>
+      </c>
+      <c r="J3" s="31">
+        <f>_xlfn.STDEV.S(D7:D11)</f>
+        <v>8.6279411698050139E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13">
+        <v>3.1376868445215297E-2</v>
+      </c>
+      <c r="C4" s="15">
+        <f t="shared" si="0"/>
+        <v>7.8442171113038243E-3</v>
+      </c>
+      <c r="D4" s="13">
+        <v>7.2078130573927882E-2</v>
+      </c>
+      <c r="F4" s="29">
+        <v>3</v>
+      </c>
+      <c r="G4" s="30">
+        <f>AVERAGE(B12:B16)</f>
+        <v>3.2684813425521146E-2</v>
+      </c>
+      <c r="H4" s="31">
+        <f>_xlfn.STDEV.S(B12:B16)</f>
+        <v>7.4399354933621627E-3</v>
+      </c>
+      <c r="I4" s="31">
+        <f>AVERAGE(D12:D16)</f>
+        <v>1.8614716917176994E-2</v>
+      </c>
+      <c r="J4" s="31">
+        <f>_xlfn.STDEV.S(D12:D16)</f>
+        <v>2.3498980955952407E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="13">
+        <v>3.3704957823215677E-2</v>
+      </c>
+      <c r="C5" s="15">
+        <f t="shared" si="0"/>
+        <v>8.4262394558039192E-3</v>
+      </c>
+      <c r="D5" s="13">
+        <v>3.7294720137639167E-2</v>
+      </c>
+      <c r="F5" s="29">
+        <v>4</v>
+      </c>
+      <c r="G5" s="30">
+        <f>AVERAGE(B17:B21)</f>
+        <v>2.5482710759610682E-2</v>
+      </c>
+      <c r="H5" s="31">
+        <f>_xlfn.STDEV.S(B17:B21)</f>
+        <v>1.3258531139342861E-2</v>
+      </c>
+      <c r="I5" s="31">
+        <f>AVERAGE(D17:D21)</f>
+        <v>2.5856802668255303E-2</v>
+      </c>
+      <c r="J5" s="31">
+        <f>_xlfn.STDEV.S(D17:D21)</f>
+        <v>1.6379127367476543E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
+        <v>1</v>
+      </c>
+      <c r="B6" s="14">
+        <v>1.422919547606802E-2</v>
+      </c>
+      <c r="C6" s="20">
+        <f>B6/4</f>
+        <v>3.557298869017005E-3</v>
+      </c>
+      <c r="D6" s="14">
+        <v>4.0868497769095208E-2</v>
+      </c>
+      <c r="F6" s="29">
+        <v>5</v>
+      </c>
+      <c r="G6" s="30">
+        <f>AVERAGE(B22:B26)</f>
+        <v>2.6401841783859431E-2</v>
+      </c>
+      <c r="H6" s="31">
+        <f>_xlfn.STDEV.S(B22:B26)</f>
+        <v>1.3442279781059763E-2</v>
+      </c>
+      <c r="I6" s="31">
+        <f>AVERAGE(D22:D26)</f>
+        <v>1.97138026162944E-2</v>
+      </c>
+      <c r="J6" s="31">
+        <f>_xlfn.STDEV.S(D22:D26)</f>
+        <v>1.7939816433876168E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="23">
+        <v>2</v>
+      </c>
+      <c r="B7" s="24">
+        <v>4.5608199354003433E-2</v>
+      </c>
+      <c r="C7" s="25">
+        <f t="shared" si="0"/>
+        <v>1.1402049838500858E-2</v>
+      </c>
+      <c r="D7" s="24">
+        <v>1.4230563740411991E-3</v>
+      </c>
+      <c r="F7" s="29">
+        <v>6</v>
+      </c>
+      <c r="G7" s="30">
+        <f>AVERAGE(B27:B31)</f>
+        <v>3.1223962225191738E-2</v>
+      </c>
+      <c r="H7" s="31">
+        <f>_xlfn.STDEV.S(B27:B31)</f>
+        <v>6.5740352445915621E-3</v>
+      </c>
+      <c r="I7" s="31">
+        <f>AVERAGE(D27:D31)</f>
+        <v>2.1684021555317776E-2</v>
+      </c>
+      <c r="J7" s="31">
+        <f>_xlfn.STDEV.S(D27:D31)</f>
+        <v>1.8808717125419688E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="23">
+        <v>2</v>
+      </c>
+      <c r="B8" s="24">
+        <v>5.4571198489538723E-2</v>
+      </c>
+      <c r="C8" s="25">
+        <f t="shared" si="0"/>
+        <v>1.3642799622384681E-2</v>
+      </c>
+      <c r="D8" s="24">
+        <v>1.751868723559423E-2</v>
+      </c>
+      <c r="F8" s="29">
+        <v>7</v>
+      </c>
+      <c r="G8" s="30">
+        <f>AVERAGE(B32:B36)</f>
+        <v>2.5991637045897943E-2</v>
+      </c>
+      <c r="H8" s="31">
+        <f>_xlfn.STDEV.S(B32:B36)</f>
+        <v>1.065847971187097E-2</v>
+      </c>
+      <c r="I8" s="31">
+        <f>AVERAGE(D32:D36)</f>
+        <v>3.7487680701257006E-2</v>
+      </c>
+      <c r="J8" s="31">
+        <f>_xlfn.STDEV.S(D32:D36)</f>
+        <v>3.5726224882368221E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="23">
+        <v>2</v>
+      </c>
+      <c r="B9" s="24">
+        <v>3.742670869175764E-2</v>
+      </c>
+      <c r="C9" s="25">
+        <f t="shared" si="0"/>
+        <v>9.3566771729394101E-3</v>
+      </c>
+      <c r="D9" s="24">
+        <v>7.6020497194364727E-3</v>
+      </c>
+      <c r="F9" s="29">
+        <v>8</v>
+      </c>
+      <c r="G9" s="30">
+        <f>AVERAGE(B37:B41)</f>
+        <v>2.6117634041361953E-2</v>
+      </c>
+      <c r="H9" s="31">
+        <f>_xlfn.STDEV.S(B37:B41)</f>
+        <v>1.047637240112336E-2</v>
+      </c>
+      <c r="I9" s="31">
+        <f>AVERAGE(D37:D41)</f>
+        <v>4.488864525301467E-2</v>
+      </c>
+      <c r="J9" s="31">
+        <f>_xlfn.STDEV.S(D37:D41)</f>
+        <v>4.8291675226136706E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="23">
+        <v>2</v>
+      </c>
+      <c r="B10" s="24">
+        <v>2.859601369462747E-2</v>
+      </c>
+      <c r="C10" s="25">
+        <f t="shared" si="0"/>
+        <v>7.1490034236568675E-3</v>
+      </c>
+      <c r="D10" s="24">
+        <v>2.1292026621170669E-2</v>
+      </c>
+      <c r="F10" s="29">
+        <v>9</v>
+      </c>
+      <c r="G10" s="30">
+        <f>AVERAGE(B42:B46)</f>
+        <v>2.6657339693028213E-2</v>
+      </c>
+      <c r="H10" s="31">
+        <f>_xlfn.STDEV.S(B42:B46)</f>
+        <v>9.5736147645614847E-3</v>
+      </c>
+      <c r="I10" s="31">
+        <f>AVERAGE(D42:D46)</f>
+        <v>3.4705696808748313E-2</v>
+      </c>
+      <c r="J10" s="31">
+        <f>_xlfn.STDEV.S(D42:D46)</f>
+        <v>2.9395927857413684E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="26">
+        <v>2</v>
+      </c>
+      <c r="B11" s="27">
+        <v>2.9459338938626241E-2</v>
+      </c>
+      <c r="C11" s="28">
+        <f t="shared" si="0"/>
+        <v>7.3648347346565602E-3</v>
+      </c>
+      <c r="D11" s="27">
+        <v>1.984571948740271E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>3</v>
+      </c>
+      <c r="B12" s="12">
+        <v>3.9444228917353122E-2</v>
+      </c>
+      <c r="C12" s="15">
+        <f t="shared" si="0"/>
+        <v>9.8610572293382805E-3</v>
+      </c>
+      <c r="D12" s="12">
+        <v>2.0886314429709001E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="6">
+        <v>3</v>
+      </c>
+      <c r="B13" s="13">
+        <v>3.824192411171274E-2</v>
+      </c>
+      <c r="C13" s="15">
+        <f t="shared" si="0"/>
+        <v>9.560481027928185E-3</v>
+      </c>
+      <c r="D13" s="13">
+        <v>1.3718770833639289E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="6">
+        <v>3</v>
+      </c>
+      <c r="B14" s="13">
+        <v>3.6339867604532769E-2</v>
+      </c>
+      <c r="C14" s="15">
+        <f t="shared" si="0"/>
+        <v>9.0849669011331922E-3</v>
+      </c>
+      <c r="D14" s="13">
+        <v>4.932531901753078E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="6">
+        <v>3</v>
+      </c>
+      <c r="B15" s="13">
+        <v>2.610156968288924E-2</v>
+      </c>
+      <c r="C15" s="15">
+        <f t="shared" si="0"/>
+        <v>6.5253924207223099E-3</v>
+      </c>
+      <c r="D15" s="13">
+        <v>5.5095178487365157E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="8">
+        <v>3</v>
+      </c>
+      <c r="B16" s="14">
+        <v>2.329647681111786E-2</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="0"/>
+        <v>5.8241192027794651E-3</v>
+      </c>
+      <c r="D16" s="14">
+        <v>2.95853656704319E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>4</v>
+      </c>
+      <c r="B17" s="12">
+        <v>3.523422680475434E-2</v>
+      </c>
+      <c r="C17" s="15">
+        <f t="shared" si="0"/>
+        <v>8.808556701188585E-3</v>
+      </c>
+      <c r="D17" s="12">
+        <v>5.8640441430261392E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="6">
+        <v>4</v>
+      </c>
+      <c r="B18" s="13">
+        <v>3.5617895391070138E-2</v>
+      </c>
+      <c r="C18" s="15">
+        <f t="shared" si="0"/>
+        <v>8.9044738477675345E-3</v>
+      </c>
+      <c r="D18" s="13">
+        <v>3.3362534037699371E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="6">
+        <v>4</v>
+      </c>
+      <c r="B19" s="13">
+        <v>3.4076437192012907E-2</v>
+      </c>
+      <c r="C19" s="15">
+        <f t="shared" si="0"/>
+        <v>8.5191092980032267E-3</v>
+      </c>
+      <c r="D19" s="13">
+        <v>1.217945838324665E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="6">
+        <v>4</v>
+      </c>
+      <c r="B20" s="13">
+        <v>1.484257088828307E-2</v>
+      </c>
+      <c r="C20" s="15">
+        <f t="shared" si="0"/>
+        <v>3.7106427220707674E-3</v>
+      </c>
+      <c r="D20" s="13">
+        <v>3.2317057276615248E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="8">
+        <v>4</v>
+      </c>
+      <c r="B21" s="14">
+        <v>7.6424235219329541E-3</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="0"/>
+        <v>1.9106058804832385E-3</v>
+      </c>
+      <c r="D21" s="14">
+        <v>4.5560919500689107E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>5</v>
+      </c>
+      <c r="B22" s="12">
+        <v>3.6102106059594671E-2</v>
+      </c>
+      <c r="C22" s="15">
+        <f t="shared" si="0"/>
+        <v>9.0255265148986678E-3</v>
+      </c>
+      <c r="D22" s="12">
+        <v>4.4746418264825939E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="6">
+        <v>5</v>
+      </c>
+      <c r="B23" s="13">
+        <v>3.6140015426741529E-2</v>
+      </c>
+      <c r="C23" s="15">
+        <f t="shared" si="0"/>
+        <v>9.0350038566853821E-3</v>
+      </c>
+      <c r="D23" s="13">
+        <v>1.1762136731325531E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="6">
+        <v>5</v>
+      </c>
+      <c r="B24" s="13">
+        <v>3.6362696049238051E-2</v>
+      </c>
+      <c r="C24" s="15">
+        <f t="shared" si="0"/>
+        <v>9.0906740123095128E-3</v>
+      </c>
+      <c r="D24" s="13">
+        <v>4.3581664033486523E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="6">
+        <v>5</v>
+      </c>
+      <c r="B25" s="13">
+        <v>1.281453147188211E-2</v>
+      </c>
+      <c r="C25" s="15">
+        <f t="shared" si="0"/>
+        <v>3.2036328679705276E-3</v>
+      </c>
+      <c r="D25" s="13">
+        <v>4.155380038366778E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="8">
+        <v>5</v>
+      </c>
+      <c r="B26" s="14">
+        <v>1.0589859911840801E-2</v>
+      </c>
+      <c r="C26" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6474649779602002E-3</v>
+      </c>
+      <c r="D26" s="14">
+        <v>3.6420267736647451E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>6</v>
+      </c>
+      <c r="B27" s="12">
+        <v>3.489256247444128E-2</v>
+      </c>
+      <c r="C27" s="15">
+        <f t="shared" si="0"/>
+        <v>8.72314061861032E-3</v>
+      </c>
+      <c r="D27" s="12">
+        <v>9.4986091852781868E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="6">
+        <v>6</v>
+      </c>
+      <c r="B28" s="13">
+        <v>3.5113982047452821E-2</v>
+      </c>
+      <c r="C28" s="15">
+        <f t="shared" si="0"/>
+        <v>8.7784955118632053E-3</v>
+      </c>
+      <c r="D28" s="13">
+        <v>2.6069073081428449E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="6">
+        <v>6</v>
+      </c>
+      <c r="B29" s="13">
+        <v>3.7773399072616419E-2</v>
+      </c>
+      <c r="C29" s="15">
+        <f t="shared" si="0"/>
+        <v>9.4433497681541047E-3</v>
+      </c>
+      <c r="D29" s="13">
+        <v>2.548648720092079E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="6">
+        <v>6</v>
+      </c>
+      <c r="B30" s="13">
+        <v>2.5136142218850629E-2</v>
+      </c>
+      <c r="C30" s="15">
+        <f t="shared" si="0"/>
+        <v>6.2840355547126572E-3</v>
+      </c>
+      <c r="D30" s="13">
+        <v>5.1252028769149569E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="8">
+        <v>6</v>
+      </c>
+      <c r="B31" s="14">
+        <v>2.320372531259755E-2</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="0"/>
+        <v>5.8009313281493875E-3</v>
+      </c>
+      <c r="D31" s="14">
+        <v>1.905174802064059E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>7</v>
+      </c>
+      <c r="B32" s="12">
+        <v>3.3607277285332221E-2</v>
+      </c>
+      <c r="C32" s="15">
+        <f t="shared" si="0"/>
+        <v>8.4018193213330553E-3</v>
+      </c>
+      <c r="D32" s="12">
+        <v>8.1683753676376654E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="6">
+        <v>7</v>
+      </c>
+      <c r="B33" s="13">
+        <v>3.6578111403873827E-2</v>
+      </c>
+      <c r="C33" s="15">
+        <f t="shared" si="0"/>
+        <v>9.1445278509684567E-3</v>
+      </c>
+      <c r="D33" s="13">
+        <v>1.105345823939813E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="6">
+        <v>7</v>
+      </c>
+      <c r="B34" s="13">
+        <v>3.003851293461552E-2</v>
+      </c>
+      <c r="C34" s="15">
+        <f t="shared" si="0"/>
+        <v>7.5096282336538801E-3</v>
+      </c>
+      <c r="D34" s="13">
+        <v>9.6822739482970252E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="6">
+        <v>7</v>
+      </c>
+      <c r="B35" s="13">
+        <v>1.1669068148248951E-2</v>
+      </c>
+      <c r="C35" s="15">
+        <f t="shared" si="0"/>
+        <v>2.9172670370622377E-3</v>
+      </c>
+      <c r="D35" s="13">
+        <v>3.8859185930349649E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="8">
+        <v>7</v>
+      </c>
+      <c r="B36" s="14">
+        <v>1.8065215457419199E-2</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" si="0"/>
+        <v>4.5163038643547997E-3</v>
+      </c>
+      <c r="D36" s="14">
+        <v>3.2534644485929347E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>8</v>
+      </c>
+      <c r="B37" s="12">
+        <v>3.5026141383485948E-2</v>
+      </c>
+      <c r="C37" s="15">
+        <f t="shared" si="0"/>
+        <v>8.756535345871487E-3</v>
+      </c>
+      <c r="D37" s="12">
+        <v>9.2490421238346741E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
+        <v>8</v>
+      </c>
+      <c r="B38" s="13">
+        <v>3.5164530967729028E-2</v>
+      </c>
+      <c r="C38" s="15">
+        <f t="shared" si="0"/>
+        <v>8.7911327419322571E-3</v>
+      </c>
+      <c r="D38" s="13">
+        <v>1.6887159468723541E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="6">
+        <v>8</v>
+      </c>
+      <c r="B39" s="13">
+        <v>3.0511145187334759E-2</v>
+      </c>
+      <c r="C39" s="15">
+        <f t="shared" si="0"/>
+        <v>7.6277862968336897E-3</v>
+      </c>
+      <c r="D39" s="13">
+        <v>0.12876312892675071</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="6">
+        <v>8</v>
+      </c>
+      <c r="B40" s="13">
+        <v>1.284917091438151E-2</v>
+      </c>
+      <c r="C40" s="15">
+        <f t="shared" si="0"/>
+        <v>3.2122927285953774E-3</v>
+      </c>
+      <c r="D40" s="13">
+        <v>3.8922545658453538E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="8">
+        <v>8</v>
+      </c>
+      <c r="B41" s="14">
+        <v>1.7037181753878521E-2</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="0"/>
+        <v>4.2592954384696301E-3</v>
+      </c>
+      <c r="D41" s="14">
+        <v>3.0621350087310869E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>9</v>
+      </c>
+      <c r="B42" s="12">
+        <v>3.371622569255172E-2</v>
+      </c>
+      <c r="C42" s="15">
+        <f t="shared" si="0"/>
+        <v>8.42905642313793E-3</v>
+      </c>
+      <c r="D42" s="12">
+        <v>8.0774734854602882E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="6">
+        <v>9</v>
+      </c>
+      <c r="B43" s="13">
+        <v>3.4941336281717653E-2</v>
+      </c>
+      <c r="C43" s="15">
+        <f t="shared" si="0"/>
+        <v>8.7353340704294132E-3</v>
+      </c>
+      <c r="D43" s="13">
+        <v>1.99072320562542E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="6">
+        <v>9</v>
+      </c>
+      <c r="B44" s="13">
+        <v>2.9813026460568451E-2</v>
+      </c>
+      <c r="C44" s="15">
+        <f t="shared" si="0"/>
+        <v>7.4532566151421127E-3</v>
+      </c>
+      <c r="D44" s="13">
+        <v>8.099305573390593E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="6">
+        <v>9</v>
+      </c>
+      <c r="B45" s="13">
+        <v>1.1615515221347929E-2</v>
+      </c>
+      <c r="C45" s="15">
+        <f t="shared" si="0"/>
+        <v>2.9038788053369824E-3</v>
+      </c>
+      <c r="D45" s="13">
+        <v>4.5951852256868868E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="8">
+        <v>9</v>
+      </c>
+      <c r="B46" s="14">
+        <v>2.320059480895531E-2</v>
+      </c>
+      <c r="C46" s="20">
+        <f t="shared" si="0"/>
+        <v>5.8001487022388276E-3</v>
+      </c>
+      <c r="D46" s="14">
+        <v>1.859887051125229E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>